<commit_message>
Temperature control from gcode and manual
Setting temperature from gcode and manual are different
</commit_message>
<xml_diff>
--- a/Calculations/J5 Angle.xlsx
+++ b/Calculations/J5 Angle.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\justi\Documents\GitHub\RA3D\Calculations\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{05DE1860-8B82-4A04-A1DB-D478EC50591B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7953D00D-E012-4D98-AE74-79E2CDE26D8E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3" uniqueCount="3">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
   <si>
     <t>Reported</t>
   </si>
@@ -45,6 +45,15 @@
   </si>
   <si>
     <t>Error</t>
+  </si>
+  <si>
+    <t>Reported2</t>
+  </si>
+  <si>
+    <t>Actual2</t>
+  </si>
+  <si>
+    <t>Error2</t>
   </si>
 </sst>
 </file>
@@ -362,10 +371,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C12"/>
+  <dimension ref="A1:F12"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="4" max="4" width="10.88671875" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -375,8 +387,17 @@
       <c r="C1" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>0</v>
       </c>
@@ -387,8 +408,18 @@
         <f>A2-B2</f>
         <v>-14.1</v>
       </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D2">
+        <v>0</v>
+      </c>
+      <c r="E2">
+        <v>0.2</v>
+      </c>
+      <c r="F2">
+        <f>D2-E2</f>
+        <v>-0.2</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>-49.84</v>
       </c>
@@ -399,8 +430,18 @@
         <f>A3-B3</f>
         <v>-21.140000000000004</v>
       </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D3">
+        <v>-3</v>
+      </c>
+      <c r="E3">
+        <v>-1.5</v>
+      </c>
+      <c r="F3">
+        <f t="shared" ref="F3:F11" si="0">D3-E3</f>
+        <v>-1.5</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>-69.968000000000004</v>
       </c>
@@ -408,11 +449,21 @@
         <v>-48</v>
       </c>
       <c r="C4">
-        <f t="shared" ref="C4:C14" si="0">A4-B4</f>
+        <f t="shared" ref="C4:C12" si="1">A4-B4</f>
         <v>-21.968000000000004</v>
       </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D4">
+        <v>-5</v>
+      </c>
+      <c r="E4">
+        <v>-4.5</v>
+      </c>
+      <c r="F4">
+        <f t="shared" si="0"/>
+        <v>-0.5</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>-10.178000000000001</v>
       </c>
@@ -420,11 +471,21 @@
         <v>3.8</v>
       </c>
       <c r="C5">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>-13.978000000000002</v>
       </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D5">
+        <v>-30</v>
+      </c>
+      <c r="E5">
+        <v>-28.5</v>
+      </c>
+      <c r="F5">
+        <f t="shared" si="0"/>
+        <v>-1.5</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>-20</v>
       </c>
@@ -432,11 +493,21 @@
         <v>0.8</v>
       </c>
       <c r="C6">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>-20.8</v>
       </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D6">
+        <v>30</v>
+      </c>
+      <c r="E6">
+        <v>24.4</v>
+      </c>
+      <c r="F6">
+        <f t="shared" si="0"/>
+        <v>5.6000000000000014</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>-20</v>
       </c>
@@ -444,11 +515,21 @@
         <v>1</v>
       </c>
       <c r="C7">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>-21</v>
       </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D7">
+        <v>-30</v>
+      </c>
+      <c r="E7">
+        <v>-28.15</v>
+      </c>
+      <c r="F7">
+        <f t="shared" si="0"/>
+        <v>-1.8500000000000014</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A8">
         <v>-30</v>
       </c>
@@ -456,11 +537,21 @@
         <v>-8.6</v>
       </c>
       <c r="C8">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>-21.4</v>
       </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D8">
+        <v>-40</v>
+      </c>
+      <c r="E8">
+        <v>-37.5</v>
+      </c>
+      <c r="F8">
+        <f t="shared" si="0"/>
+        <v>-2.5</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A9">
         <v>-40</v>
       </c>
@@ -468,11 +559,21 @@
         <v>-18.2</v>
       </c>
       <c r="C9">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>-21.8</v>
       </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D9">
+        <v>-50</v>
+      </c>
+      <c r="E9">
+        <v>-47.5</v>
+      </c>
+      <c r="F9">
+        <f t="shared" si="0"/>
+        <v>-2.5</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A10">
         <v>-50</v>
       </c>
@@ -480,11 +581,21 @@
         <v>-28</v>
       </c>
       <c r="C10">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>-22</v>
       </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D10">
+        <v>-60</v>
+      </c>
+      <c r="E10">
+        <v>-56.2</v>
+      </c>
+      <c r="F10">
+        <f t="shared" si="0"/>
+        <v>-3.7999999999999972</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A11">
         <v>40</v>
       </c>
@@ -492,11 +603,21 @@
         <v>54</v>
       </c>
       <c r="C11">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>-14</v>
       </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D11">
+        <v>-55</v>
+      </c>
+      <c r="E11">
+        <v>-56.2</v>
+      </c>
+      <c r="F11">
+        <f t="shared" si="0"/>
+        <v>1.2000000000000028</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A12">
         <v>50</v>
       </c>
@@ -504,7 +625,7 @@
         <v>63</v>
       </c>
       <c r="C12">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>-13</v>
       </c>
     </row>

</xml_diff>